<commit_message>
Add ECE cluster benchmark results
</commit_message>
<xml_diff>
--- a/results/large_integer_multiplication_charts.xlsx
+++ b/results/large_integer_multiplication_charts.xlsx
@@ -824,17 +824,21 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="n"/>
+      <c r="B2" s="3" t="n">
+        <v>1114206.128</v>
+      </c>
       <c r="C2" s="3" t="n">
         <v>980392.1568999999</v>
       </c>
-      <c r="D2" s="3" t="n"/>
+      <c r="D2" s="3" t="n">
+        <v>3497668.221</v>
+      </c>
       <c r="E2" s="3" t="n">
         <v>4361370.717</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Paste ECE flops/s values into columns B and D.</t>
+          <t>Source files: aws_ec2_multiply_benchmark.csv and ece_cluster_multiply_benchmark.csv.</t>
         </is>
       </c>
     </row>
@@ -842,17 +846,21 @@
       <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="n"/>
+      <c r="B3" s="3" t="n">
+        <v>29411764.71</v>
+      </c>
       <c r="C3" s="3" t="n">
         <v>33333333.33</v>
       </c>
-      <c r="D3" s="3" t="n"/>
+      <c r="D3" s="3" t="n">
+        <v>154506437.8</v>
+      </c>
       <c r="E3" s="3" t="n">
         <v>163636363.6</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>The two chart sheets update automatically in Excel.</t>
+          <t>Each chart contains ECE Cluster and AWS EC2 clustered columns.</t>
         </is>
       </c>
     </row>
@@ -860,11 +868,15 @@
       <c r="A4" t="n">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="n"/>
+      <c r="B4" s="3" t="n">
+        <v>110726643.6</v>
+      </c>
       <c r="C4" s="3" t="n">
         <v>168421052.6</v>
       </c>
-      <c r="D4" s="3" t="n"/>
+      <c r="D4" s="3" t="n">
+        <v>327710843.4</v>
+      </c>
       <c r="E4" s="3" t="n">
         <v>412121212.1</v>
       </c>
@@ -873,11 +885,15 @@
       <c r="A5" t="n">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="n"/>
+      <c r="B5" s="3" t="n">
+        <v>486692015.2</v>
+      </c>
       <c r="C5" s="3" t="n">
         <v>556521739.1</v>
       </c>
-      <c r="D5" s="3" t="n"/>
+      <c r="D5" s="3" t="n">
+        <v>609699769.1</v>
+      </c>
       <c r="E5" s="3" t="n">
         <v>759712230.2</v>
       </c>
@@ -886,11 +902,15 @@
       <c r="A6" t="n">
         <v>16</v>
       </c>
-      <c r="B6" s="3" t="n"/>
+      <c r="B6" s="3" t="n">
+        <v>1028112450</v>
+      </c>
       <c r="C6" s="3" t="n">
         <v>1383783784</v>
       </c>
-      <c r="D6" s="3" t="n"/>
+      <c r="D6" s="3" t="n">
+        <v>858562437.9</v>
+      </c>
       <c r="E6" s="3" t="n">
         <v>1216901408</v>
       </c>
@@ -899,11 +919,15 @@
       <c r="A7" t="n">
         <v>32</v>
       </c>
-      <c r="B7" s="3" t="n"/>
+      <c r="B7" s="3" t="n">
+        <v>3255961844</v>
+      </c>
       <c r="C7" s="3" t="n">
         <v>3592982456</v>
       </c>
-      <c r="D7" s="3" t="n"/>
+      <c r="D7" s="3" t="n">
+        <v>970309538.9</v>
+      </c>
       <c r="E7" s="3" t="n">
         <v>1154887218</v>
       </c>
@@ -912,11 +936,15 @@
       <c r="A8" t="n">
         <v>64</v>
       </c>
-      <c r="B8" s="3" t="n"/>
+      <c r="B8" s="3" t="n">
+        <v>6989761092</v>
+      </c>
       <c r="C8" s="3" t="n">
         <v>6884033613</v>
       </c>
-      <c r="D8" s="3" t="n"/>
+      <c r="D8" s="3" t="n">
+        <v>1555677214</v>
+      </c>
       <c r="E8" s="3" t="n">
         <v>1911990311</v>
       </c>
@@ -925,11 +953,15 @@
       <c r="A9" t="n">
         <v>128</v>
       </c>
-      <c r="B9" s="3" t="n"/>
+      <c r="B9" s="3" t="n">
+        <v>10900864940</v>
+      </c>
       <c r="C9" s="3" t="n">
         <v>12951778660</v>
       </c>
-      <c r="D9" s="3" t="n"/>
+      <c r="D9" s="3" t="n">
+        <v>1913280740</v>
+      </c>
       <c r="E9" s="3" t="n">
         <v>2672410936</v>
       </c>
@@ -938,11 +970,15 @@
       <c r="A10" t="n">
         <v>256</v>
       </c>
-      <c r="B10" s="3" t="n"/>
+      <c r="B10" s="3" t="n">
+        <v>12968437720</v>
+      </c>
       <c r="C10" s="3" t="n">
         <v>21736650080</v>
       </c>
-      <c r="D10" s="3" t="n"/>
+      <c r="D10" s="3" t="n">
+        <v>2107857164</v>
+      </c>
       <c r="E10" s="3" t="n">
         <v>3001746362</v>
       </c>
@@ -951,11 +987,15 @@
       <c r="A11" t="n">
         <v>512</v>
       </c>
-      <c r="B11" s="3" t="n"/>
+      <c r="B11" s="3" t="n">
+        <v>15258228810</v>
+      </c>
       <c r="C11" s="3" t="n">
         <v>26845263700</v>
       </c>
-      <c r="D11" s="3" t="n"/>
+      <c r="D11" s="3" t="n">
+        <v>1862339116</v>
+      </c>
       <c r="E11" s="3" t="n">
         <v>3004400978</v>
       </c>
@@ -964,11 +1004,15 @@
       <c r="A12" t="n">
         <v>1024</v>
       </c>
-      <c r="B12" s="3" t="n"/>
+      <c r="B12" s="3" t="n">
+        <v>16278318110</v>
+      </c>
       <c r="C12" s="3" t="n">
         <v>30736058390</v>
       </c>
-      <c r="D12" s="3" t="n"/>
+      <c r="D12" s="3" t="n">
+        <v>2218345590</v>
+      </c>
       <c r="E12" s="3" t="n">
         <v>3211149826</v>
       </c>
@@ -977,11 +1021,15 @@
       <c r="A13" t="n">
         <v>2048</v>
       </c>
-      <c r="B13" s="3" t="n"/>
+      <c r="B13" s="3" t="n">
+        <v>16649580320</v>
+      </c>
       <c r="C13" s="3" t="n">
         <v>32659432900</v>
       </c>
-      <c r="D13" s="3" t="n"/>
+      <c r="D13" s="3" t="n">
+        <v>1895282045</v>
+      </c>
       <c r="E13" s="3" t="n">
         <v>3184590690</v>
       </c>
@@ -990,11 +1038,15 @@
       <c r="A14" t="n">
         <v>4096</v>
       </c>
-      <c r="B14" s="3" t="n"/>
+      <c r="B14" s="3" t="n">
+        <v>16638203810</v>
+      </c>
       <c r="C14" s="3" t="n">
         <v>33308449100</v>
       </c>
-      <c r="D14" s="3" t="n"/>
+      <c r="D14" s="3" t="n">
+        <v>1715400130</v>
+      </c>
       <c r="E14" s="3" t="n">
         <v>2987491881</v>
       </c>
@@ -1003,11 +1055,15 @@
       <c r="A15" t="n">
         <v>8192</v>
       </c>
-      <c r="B15" s="3" t="n"/>
+      <c r="B15" s="3" t="n">
+        <v>16252257910</v>
+      </c>
       <c r="C15" s="3" t="n">
         <v>30822467210</v>
       </c>
-      <c r="D15" s="3" t="n"/>
+      <c r="D15" s="3" t="n">
+        <v>2030460255</v>
+      </c>
       <c r="E15" s="3" t="n">
         <v>3078560648</v>
       </c>
@@ -1016,11 +1072,15 @@
       <c r="A16" t="n">
         <v>16384</v>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="3" t="n">
+        <v>16233858120</v>
+      </c>
       <c r="C16" s="3" t="n">
         <v>30853880540</v>
       </c>
-      <c r="D16" s="3" t="n"/>
+      <c r="D16" s="3" t="n">
+        <v>2061099918</v>
+      </c>
       <c r="E16" s="3" t="n">
         <v>3083246844</v>
       </c>
@@ -1029,11 +1089,15 @@
       <c r="A17" t="n">
         <v>32768</v>
       </c>
-      <c r="B17" s="3" t="n"/>
+      <c r="B17" s="3" t="n">
+        <v>16796434010</v>
+      </c>
       <c r="C17" s="3" t="n">
         <v>31158053900</v>
       </c>
-      <c r="D17" s="3" t="n"/>
+      <c r="D17" s="3" t="n">
+        <v>2041694918</v>
+      </c>
       <c r="E17" s="3" t="n">
         <v>3111351362</v>
       </c>
@@ -1042,11 +1106,15 @@
       <c r="A18" t="n">
         <v>65536</v>
       </c>
-      <c r="B18" s="3" t="n"/>
+      <c r="B18" s="3" t="n">
+        <v>16897101930</v>
+      </c>
       <c r="C18" s="3" t="n">
         <v>31352435230</v>
       </c>
-      <c r="D18" s="3" t="n"/>
+      <c r="D18" s="3" t="n">
+        <v>2069289250</v>
+      </c>
       <c r="E18" s="3" t="n">
         <v>3174465156</v>
       </c>
@@ -1055,11 +1123,15 @@
       <c r="A19" t="n">
         <v>131072</v>
       </c>
-      <c r="B19" s="3" t="n"/>
+      <c r="B19" s="3" t="n">
+        <v>17012342780</v>
+      </c>
       <c r="C19" s="3" t="n">
         <v>31074076650</v>
       </c>
-      <c r="D19" s="3" t="n"/>
+      <c r="D19" s="3" t="n">
+        <v>2126013902</v>
+      </c>
       <c r="E19" s="3" t="n">
         <v>3220380767</v>
       </c>
@@ -1068,11 +1140,15 @@
       <c r="A20" t="n">
         <v>262144</v>
       </c>
-      <c r="B20" s="3" t="n"/>
+      <c r="B20" s="3" t="n">
+        <v>12415845500</v>
+      </c>
       <c r="C20" s="3" t="n">
         <v>28907155820</v>
       </c>
-      <c r="D20" s="3" t="n"/>
+      <c r="D20" s="3" t="n">
+        <v>2057014043</v>
+      </c>
       <c r="E20" s="3" t="n">
         <v>3236511205</v>
       </c>
@@ -1081,11 +1157,15 @@
       <c r="A21" t="n">
         <v>524288</v>
       </c>
-      <c r="B21" s="3" t="n"/>
+      <c r="B21" s="3" t="n">
+        <v>11340743640</v>
+      </c>
       <c r="C21" s="3" t="n">
         <v>29309315220</v>
       </c>
-      <c r="D21" s="3" t="n"/>
+      <c r="D21" s="3" t="n">
+        <v>1768690284</v>
+      </c>
       <c r="E21" s="3" t="n">
         <v>3098819079</v>
       </c>
@@ -1094,11 +1174,15 @@
       <c r="A22" t="n">
         <v>1048576</v>
       </c>
-      <c r="B22" s="3" t="n"/>
+      <c r="B22" s="3" t="n">
+        <v>10720188860</v>
+      </c>
       <c r="C22" s="3" t="n">
         <v>29341832210</v>
       </c>
-      <c r="D22" s="3" t="n"/>
+      <c r="D22" s="3" t="n">
+        <v>1653164747</v>
+      </c>
       <c r="E22" s="3" t="n">
         <v>2725606636</v>
       </c>
@@ -1107,11 +1191,15 @@
       <c r="A23" t="n">
         <v>2097152</v>
       </c>
-      <c r="B23" s="3" t="n"/>
+      <c r="B23" s="3" t="n">
+        <v>10462847460</v>
+      </c>
       <c r="C23" s="3" t="n">
         <v>29258605910</v>
       </c>
-      <c r="D23" s="3" t="n"/>
+      <c r="D23" s="3" t="n">
+        <v>1532549227</v>
+      </c>
       <c r="E23" s="3" t="n">
         <v>2570118998</v>
       </c>
@@ -1140,7 +1228,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ECE Cluster data is intentionally blank until that run is available.</t>
+          <t>Clustered columns compare ECE Cluster and AWS EC2 for each input length.</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1257,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>ECE Cluster data is intentionally blank until that run is available.</t>
+          <t>Clustered columns compare ECE Cluster and AWS EC2 for each input length.</t>
         </is>
       </c>
     </row>

</xml_diff>